<commit_message>
corrected a data unit from USD to SSP
</commit_message>
<xml_diff>
--- a/data/sepi_results_v1_aligned_equal_weighted_raw_subindicators.xlsx
+++ b/data/sepi_results_v1_aligned_equal_weighted_raw_subindicators.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://undp-my.sharepoint.com/personal/ela_dogan_undp_org/Documents/Desktop/Socioeconomic-Peace-Index-Tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1C41E2E-E9F3-467A-A4F1-304E4388C8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A1C41E2E-E9F3-467A-A4F1-304E4388C8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA95FD91-9D76-480D-B0E9-D575EC2FE4DF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="453">
   <si>
     <t>Section</t>
   </si>
@@ -1398,6 +1398,9 @@
   </si>
   <si>
     <t>This pillar measures environmental conditions that affect livelihoods, food production, and population stability. It incorporates indicators such as drought severity (PDSI), vegetation health (NDVI), absorbed solar radiation (FAPAR), and soil moisture anomalies — all derived from remote sensing data. In line with the humanitarian-development-peace nexus, climate-induced stressors are recognised as compounding drivers of fragility, forced displacement, and conflict vulnerability across the Horn of Africa. A higher pillar score indicates greater socio-economic resilience in this dimension.</t>
+  </si>
+  <si>
+    <t>SSP</t>
   </si>
 </sst>
 </file>
@@ -9874,7 +9877,7 @@
         <v>363</v>
       </c>
       <c r="F37" t="s">
-        <v>353</v>
+        <v>452</v>
       </c>
       <c r="G37" t="s">
         <v>364</v>
@@ -20770,14 +20773,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="fcf89adc-eefc-4033-818a-934b0690d419" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6b197b6a-cffc-4ca7-9de0-77d82e42a5a9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21016,21 +21017,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="fcf89adc-eefc-4033-818a-934b0690d419" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6b197b6a-cffc-4ca7-9de0-77d82e42a5a9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{471C6B65-D68C-40D5-A1A2-6C3F7EBAAC65}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87A03265-2C13-4CBB-A0BE-0F46518CCCA1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fcf89adc-eefc-4033-818a-934b0690d419"/>
-    <ds:schemaRef ds:uri="6b197b6a-cffc-4ca7-9de0-77d82e42a5a9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -21055,9 +21055,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87A03265-2C13-4CBB-A0BE-0F46518CCCA1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{471C6B65-D68C-40D5-A1A2-6C3F7EBAAC65}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fcf89adc-eefc-4033-818a-934b0690d419"/>
+    <ds:schemaRef ds:uri="6b197b6a-cffc-4ca7-9de0-77d82e42a5a9"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>